<commit_message>
TUT Cua A audit: Binance spot TUTUSDT phat hien, DAILY spot columns dien
- docs/case_files/CASE_TUT.xlsx: cap nhat 36 rows voi spot_bnb + DEX
  - vol_spot_usd: Binance spot + BSC DEX daily (09/07->04/08)
  - taker_spot_pct: Binance fapi klines taker (avg 51.1% = neutral)
  - venue_top: Binance_spot_TUTUSDT (phat hien moi - truoc gia su khong co)
  - CASE sheet: S1 venue map, spot/perp ratio 0.17x, Cua A capacity
- scratch/tut_cua_a_20260805.txt: raw probe output
- agent_log.md: S1-S4 summary

Key findings:
- Binance spot TUTUSDT LISTED (khong phai Alpha, khong phai BSC-only)
- AKE-test: spot/perp = 0.055-0.40x (trung binh 0.17x) — spot co that
- Taker spot avg 51.1%: TRUNG TINH — khong ro tin hieu phan phoi
- Cua A max capacity: $11.3M/27ngay (upper bound, PENDING O1 supply)
- S3 verdict: AMBIGUOUS — can exchange balance tu operator

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_TUT.xlsx
+++ b/docs/case_files/CASE_TUT.xlsx
@@ -22,9 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.00000"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -51,7 +52,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +84,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -96,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +116,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -475,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -496,7 +506,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -588,7 +597,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -686,7 +694,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
@@ -816,7 +823,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
@@ -857,6 +863,94 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>PENDING — Nansen LOCKED, operator feed</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>S1 VENUE DISCOVERY (05/08)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Binance spot TUTUSDT: LISTED! vol $0.23-7.16M/day. CoinGecko tickers: 24 markets (Gate/MEXC/LBank $16-84M — SUSPICIOUS wash). Alpha_117: 400 error (defunct).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>venue_top</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Binance_spot_TUTUSDT (confirmed via api.binance.com)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>spot_perp_ratio_campaign</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0.169x avg (Binance spot $30M + DEX $5M vs perp $207M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>taker_spot_avg</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>50.8% (neutral — no clear distribution signal from taker alone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>cua_A_capacity_day</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>$426k/day (30% of $1.42M avg spot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>cua_A_total_27d_max</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>$11.5M possible spot distribution in 27 days (upper bound)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>S3_verdict</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>AMBIGUOUS: taker neutral, no DEX large sell pattern visible. On-chain balance PENDING.</t>
         </is>
       </c>
     </row>
@@ -5368,12 +5462,18 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB64" t="n">
+        <v>290000</v>
+      </c>
+      <c r="AC64" s="13" t="n">
+        <v>0.52</v>
       </c>
       <c r="AO64" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -5434,12 +5534,18 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB65" t="n">
+        <v>400000</v>
+      </c>
+      <c r="AC65" s="13" t="n">
+        <v>0.524</v>
       </c>
       <c r="AO65" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -5500,12 +5606,18 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB66" t="n">
+        <v>280000</v>
+      </c>
+      <c r="AC66" s="13" t="n">
+        <v>0.644</v>
       </c>
       <c r="AO66" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -5566,12 +5678,18 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB67" t="n">
+        <v>350000</v>
+      </c>
+      <c r="AC67" s="13" t="n">
+        <v>0.522</v>
       </c>
       <c r="AO67" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -5632,12 +5750,18 @@
       </c>
       <c r="AA68" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB68" t="n">
+        <v>750000</v>
+      </c>
+      <c r="AC68" s="13" t="n">
+        <v>0.487</v>
       </c>
       <c r="AO68" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -5698,12 +5822,18 @@
       </c>
       <c r="AA69" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB69" t="n">
+        <v>650000</v>
+      </c>
+      <c r="AC69" s="13" t="n">
+        <v>0.528</v>
       </c>
       <c r="AO69" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -5764,8 +5894,14 @@
       </c>
       <c r="AA70" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB70" t="n">
+        <v>690000</v>
+      </c>
+      <c r="AC70" s="13" t="n">
+        <v>0.476</v>
       </c>
       <c r="AM70" s="11" t="n"/>
       <c r="AN70" t="inlineStr">
@@ -5775,7 +5911,7 @@
       </c>
       <c r="AO70" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -5836,8 +5972,14 @@
       </c>
       <c r="AA71" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB71" t="n">
+        <v>230000</v>
+      </c>
+      <c r="AC71" s="13" t="n">
+        <v>0.461</v>
       </c>
       <c r="AM71" s="11" t="n"/>
       <c r="AN71" t="inlineStr">
@@ -5847,7 +5989,7 @@
       </c>
       <c r="AO71" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -5908,8 +6050,14 @@
       </c>
       <c r="AA72" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB72" t="n">
+        <v>1060000</v>
+      </c>
+      <c r="AC72" s="14" t="n">
+        <v>0.548</v>
       </c>
       <c r="AM72" s="11" t="n"/>
       <c r="AN72" t="inlineStr">
@@ -5919,7 +6067,7 @@
       </c>
       <c r="AO72" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -5980,8 +6128,14 @@
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB73" t="n">
+        <v>470000</v>
+      </c>
+      <c r="AC73" s="13" t="n">
+        <v>0.57</v>
       </c>
       <c r="AM73" s="11" t="n"/>
       <c r="AN73" t="inlineStr">
@@ -5991,7 +6145,7 @@
       </c>
       <c r="AO73" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6052,12 +6206,18 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB74" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="AC74" s="14" t="n">
+        <v>0.549</v>
       </c>
       <c r="AO74" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6118,8 +6278,14 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB75" t="n">
+        <v>1030000</v>
+      </c>
+      <c r="AC75" s="13" t="n">
+        <v>0.464</v>
       </c>
       <c r="AM75" s="11" t="n"/>
       <c r="AN75" t="inlineStr">
@@ -6129,7 +6295,7 @@
       </c>
       <c r="AO75" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6190,12 +6356,18 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB76" t="n">
+        <v>610000</v>
+      </c>
+      <c r="AC76" s="13" t="n">
+        <v>0.547</v>
       </c>
       <c r="AO76" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6256,12 +6428,18 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB77" t="n">
+        <v>350000</v>
+      </c>
+      <c r="AC77" s="13" t="n">
+        <v>0.504</v>
       </c>
       <c r="AO77" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6322,12 +6500,18 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB78" t="n">
+        <v>400000</v>
+      </c>
+      <c r="AC78" s="13" t="n">
+        <v>0.479</v>
       </c>
       <c r="AO78" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6388,12 +6572,18 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB79" t="n">
+        <v>380000</v>
+      </c>
+      <c r="AC79" s="13" t="n">
+        <v>0.511</v>
       </c>
       <c r="AO79" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6454,12 +6644,18 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB80" t="n">
+        <v>510000</v>
+      </c>
+      <c r="AC80" s="13" t="n">
+        <v>0.548</v>
       </c>
       <c r="AO80" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6520,12 +6716,18 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB81" t="n">
+        <v>360000</v>
+      </c>
+      <c r="AC81" s="13" t="n">
+        <v>0.51</v>
       </c>
       <c r="AO81" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6586,12 +6788,18 @@
       </c>
       <c r="AA82" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB82" t="n">
+        <v>180000</v>
+      </c>
+      <c r="AC82" s="13" t="n">
+        <v>0.379</v>
       </c>
       <c r="AO82" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6652,12 +6860,18 @@
       </c>
       <c r="AA83" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB83" t="n">
+        <v>940000</v>
+      </c>
+      <c r="AC83" s="13" t="n">
+        <v>0.569</v>
       </c>
       <c r="AO83" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6718,12 +6932,18 @@
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB84" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="AC84" s="13" t="n">
+        <v>0.518</v>
       </c>
       <c r="AO84" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6784,12 +7004,18 @@
       </c>
       <c r="AA85" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB85" t="n">
+        <v>1030000</v>
+      </c>
+      <c r="AC85" s="13" t="n">
+        <v>0.523</v>
       </c>
       <c r="AO85" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6850,12 +7076,18 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB86" t="n">
+        <v>420000</v>
+      </c>
+      <c r="AC86" s="15" t="n">
+        <v>0.441</v>
       </c>
       <c r="AO86" t="inlineStr">
         <is>
-          <t>freshwatch/derived_1h</t>
+          <t>freshwatch/derived_1h+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6906,11 +7138,15 @@
       </c>
       <c r="AA87" s="4" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
-      </c>
-      <c r="AB87" s="4" t="n"/>
-      <c r="AC87" s="4" t="n"/>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB87" s="4" t="n">
+        <v>450000</v>
+      </c>
+      <c r="AC87" s="16" t="n">
+        <v>0.491</v>
+      </c>
       <c r="AD87" s="4" t="n"/>
       <c r="AE87" s="4" t="n"/>
       <c r="AF87" s="4" t="n"/>
@@ -6924,7 +7160,7 @@
       <c r="AN87" s="4" t="n"/>
       <c r="AO87" s="4" t="inlineStr">
         <is>
-          <t>fapi_klines_only</t>
+          <t>fapi_klines_only+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -6975,11 +7211,15 @@
       </c>
       <c r="AA88" s="4" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
-      </c>
-      <c r="AB88" s="4" t="n"/>
-      <c r="AC88" s="4" t="n"/>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB88" s="4" t="n">
+        <v>730000</v>
+      </c>
+      <c r="AC88" s="16" t="n">
+        <v>0.51</v>
+      </c>
       <c r="AD88" s="4" t="n"/>
       <c r="AE88" s="4" t="n"/>
       <c r="AF88" s="4" t="n"/>
@@ -6993,7 +7233,7 @@
       <c r="AN88" s="4" t="n"/>
       <c r="AO88" s="4" t="inlineStr">
         <is>
-          <t>fapi_klines_only</t>
+          <t>fapi_klines_only+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7044,11 +7284,15 @@
       </c>
       <c r="AA89" s="4" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
-      </c>
-      <c r="AB89" s="4" t="n"/>
-      <c r="AC89" s="4" t="n"/>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB89" s="4" t="n">
+        <v>460000</v>
+      </c>
+      <c r="AC89" s="16" t="n">
+        <v>0.492</v>
+      </c>
       <c r="AD89" s="4" t="n"/>
       <c r="AE89" s="4" t="n"/>
       <c r="AF89" s="4" t="n"/>
@@ -7062,7 +7306,7 @@
       <c r="AN89" s="4" t="n"/>
       <c r="AO89" s="4" t="inlineStr">
         <is>
-          <t>fapi_klines_only</t>
+          <t>fapi_klines_only+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7123,12 +7367,18 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB90" t="n">
+        <v>600000</v>
+      </c>
+      <c r="AC90" s="13" t="n">
+        <v>0.497</v>
       </c>
       <c r="AO90" t="inlineStr">
         <is>
-          <t>freshwatch/native_1d</t>
+          <t>freshwatch/native_1d+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7189,12 +7439,18 @@
       </c>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB91" t="n">
+        <v>930000</v>
+      </c>
+      <c r="AC91" s="13" t="n">
+        <v>0.578</v>
       </c>
       <c r="AO91" t="inlineStr">
         <is>
-          <t>freshwatch/native_1d</t>
+          <t>freshwatch/native_1d+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7255,12 +7511,18 @@
       </c>
       <c r="AA92" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB92" t="n">
+        <v>860000</v>
+      </c>
+      <c r="AC92" s="13" t="n">
+        <v>0.502</v>
       </c>
       <c r="AO92" t="inlineStr">
         <is>
-          <t>freshwatch/native_1d</t>
+          <t>freshwatch/native_1d+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7321,12 +7583,18 @@
       </c>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB93" t="n">
+        <v>420000</v>
+      </c>
+      <c r="AC93" s="13" t="n">
+        <v>0.466</v>
       </c>
       <c r="AO93" t="inlineStr">
         <is>
-          <t>freshwatch/native_1d</t>
+          <t>freshwatch/native_1d+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7387,12 +7655,18 @@
       </c>
       <c r="AA94" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB94" t="n">
+        <v>960000</v>
+      </c>
+      <c r="AC94" s="15" t="n">
+        <v>0.442</v>
       </c>
       <c r="AO94" t="inlineStr">
         <is>
-          <t>freshwatch/native_1d</t>
+          <t>freshwatch/native_1d+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7453,12 +7727,18 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB95" t="n">
+        <v>3266272</v>
+      </c>
+      <c r="AC95" s="14" t="n">
+        <v>0.542</v>
       </c>
       <c r="AO95" t="inlineStr">
         <is>
-          <t>freshwatch/native_1d</t>
+          <t>freshwatch/native_1d+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7519,8 +7799,14 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB96" t="n">
+        <v>1163961</v>
+      </c>
+      <c r="AC96" s="13" t="n">
+        <v>0.54</v>
       </c>
       <c r="AM96" s="11" t="n"/>
       <c r="AN96" t="inlineStr">
@@ -7530,7 +7816,7 @@
       </c>
       <c r="AO96" t="inlineStr">
         <is>
-          <t>freshwatch/native_1d</t>
+          <t>freshwatch/native_1d+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7591,12 +7877,18 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB97" t="n">
+        <v>6211822</v>
+      </c>
+      <c r="AC97" s="14" t="n">
+        <v>0.5679999999999999</v>
       </c>
       <c r="AO97" t="inlineStr">
         <is>
-          <t>freshwatch/native_1d</t>
+          <t>freshwatch/native_1d+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7657,8 +7949,14 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB98" t="n">
+        <v>8180835</v>
+      </c>
+      <c r="AC98" s="13" t="n">
+        <v>0.509</v>
       </c>
       <c r="AM98" s="11" t="n"/>
       <c r="AN98" t="inlineStr">
@@ -7668,7 +7966,7 @@
       </c>
       <c r="AO98" t="inlineStr">
         <is>
-          <t>freshwatch/native_1d</t>
+          <t>freshwatch/native_1d+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7723,11 +8021,15 @@
       </c>
       <c r="AA99" s="4" t="inlineStr">
         <is>
-          <t>BSC_DEX_WBNB</t>
-        </is>
-      </c>
-      <c r="AB99" s="4" t="n"/>
-      <c r="AC99" s="4" t="n"/>
+          <t>Binance_spot+BSC_DEX</t>
+        </is>
+      </c>
+      <c r="AB99" s="4" t="n">
+        <v>1479152</v>
+      </c>
+      <c r="AC99" s="15" t="n">
+        <v>0.44</v>
+      </c>
       <c r="AD99" s="4" t="n"/>
       <c r="AE99" s="4" t="n"/>
       <c r="AF99" s="4" t="n"/>
@@ -7741,7 +8043,7 @@
       <c r="AN99" s="4" t="n"/>
       <c r="AO99" s="4" t="inlineStr">
         <is>
-          <t>fapi_klines+oi_rt</t>
+          <t>fapi_klines+oi_rt+spot_klines_Binance</t>
         </is>
       </c>
     </row>
@@ -7778,7 +8080,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -8249,7 +8550,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -8432,7 +8732,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -8711,7 +9010,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -8748,7 +9046,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -8816,7 +9113,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -8888,7 +9184,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -8961,7 +9256,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>

</xml_diff>